<commit_message>
Excel-only data, multisheet parser, industrial map, Seismic
</commit_message>
<xml_diff>
--- a/data/Data_Center_Site_Selector_RH.xlsx
+++ b/data/Data_Center_Site_Selector_RH.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://colostate-my.sharepoint.com/personal/laffite_colostate_edu/Documents/Desktop/Classes/2026 Spring/CIVE-580C4 Applying AI in Environmental Engr Practice/Final project/App_v2/Siteworks2/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1129" documentId="11_CB780128D071F47F630230D6525DCE3A2746A58A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E2FC351C-6648-4776-8B04-7F63B941E772}"/>
+  <xr:revisionPtr revIDLastSave="1151" documentId="11_CB780128D071F47F630230D6525DCE3A2746A58A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{021857B9-811B-4D0E-A50C-2B3CD42429A0}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" tabRatio="707" activeTab="3" xr2:uid="{C789D543-12B0-4242-A688-B41AF874B720}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" tabRatio="707" activeTab="4" xr2:uid="{C789D543-12B0-4242-A688-B41AF874B720}"/>
   </bookViews>
   <sheets>
     <sheet name="Site Selector Data - edited" sheetId="2" r:id="rId1"/>
@@ -418,7 +418,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="173">
   <si>
     <t>Account Weights</t>
   </si>
@@ -931,6 +931,12 @@
   </si>
   <si>
     <t>Scenario</t>
+  </si>
+  <si>
+    <t>best</t>
+  </si>
+  <si>
+    <t>worst</t>
   </si>
 </sst>
 </file>
@@ -1338,7 +1344,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1487,6 +1493,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1520,15 +1535,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1544,7 +1550,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1858,7 +1863,7 @@
     <col min="5" max="5" width="8" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="8" customWidth="1"/>
-    <col min="8" max="8" width="90" customWidth="1"/>
+    <col min="8" max="8" width="90" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="42.109375" style="3" customWidth="1"/>
     <col min="11" max="11" width="11.77734375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="9.6640625" bestFit="1" customWidth="1"/>
@@ -1974,10 +1979,10 @@
       <c r="I5" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="J5" s="69" t="s">
+      <c r="J5" s="72" t="s">
         <v>163</v>
       </c>
-      <c r="K5" s="70"/>
+      <c r="K5" s="73"/>
       <c r="L5" s="16"/>
     </row>
     <row r="6" spans="1:12" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2005,7 +2010,7 @@
       <c r="H6" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="72" t="s">
+      <c r="I6" s="61" t="s">
         <v>138</v>
       </c>
       <c r="J6" s="12">
@@ -2032,7 +2037,7 @@
       <c r="H7" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="I7" s="72"/>
+      <c r="I7" s="61"/>
       <c r="J7" s="12">
         <v>4</v>
       </c>
@@ -2057,7 +2062,7 @@
       <c r="H8" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="I8" s="72"/>
+      <c r="I8" s="61"/>
       <c r="J8" s="12">
         <v>3</v>
       </c>
@@ -2082,7 +2087,7 @@
       <c r="H9" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="I9" s="72"/>
+      <c r="I9" s="61"/>
       <c r="J9" s="12">
         <v>2</v>
       </c>
@@ -2107,7 +2112,7 @@
       <c r="H10" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="I10" s="73"/>
+      <c r="I10" s="62"/>
       <c r="J10" s="13">
         <v>1</v>
       </c>
@@ -2135,19 +2140,19 @@
         <v>36.950000000000003</v>
       </c>
       <c r="G11" s="48">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H11" s="37" t="s">
         <v>35</v>
       </c>
-      <c r="I11" s="71" t="s">
+      <c r="I11" s="60" t="s">
         <v>139</v>
       </c>
       <c r="J11" s="12">
         <v>5</v>
       </c>
       <c r="K11" s="14" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
@@ -2162,12 +2167,12 @@
         <v>92.79</v>
       </c>
       <c r="G12" s="46">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H12" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="I12" s="72"/>
+      <c r="I12" s="61"/>
       <c r="J12" s="12">
         <v>4</v>
       </c>
@@ -2185,12 +2190,12 @@
         <v>56.55</v>
       </c>
       <c r="G13" s="46">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H13" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="I13" s="72"/>
+      <c r="I13" s="61"/>
       <c r="J13" s="12">
         <v>3</v>
       </c>
@@ -2213,7 +2218,7 @@
       <c r="H14" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="I14" s="72"/>
+      <c r="I14" s="61"/>
       <c r="J14" s="12">
         <v>2</v>
       </c>
@@ -2231,17 +2236,17 @@
         <v>48.31</v>
       </c>
       <c r="G15" s="47">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H15" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="I15" s="73"/>
+      <c r="I15" s="62"/>
       <c r="J15" s="13">
         <v>1</v>
       </c>
       <c r="K15" s="15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -2269,7 +2274,7 @@
       <c r="H16" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="I16" s="63" t="s">
+      <c r="I16" s="66" t="s">
         <v>140</v>
       </c>
       <c r="J16" s="12">
@@ -2296,7 +2301,7 @@
       <c r="H17" s="38" t="s">
         <v>100</v>
       </c>
-      <c r="I17" s="64"/>
+      <c r="I17" s="67"/>
       <c r="J17" s="12">
         <v>1</v>
       </c>
@@ -2321,7 +2326,7 @@
       <c r="H18" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="I18" s="64"/>
+      <c r="I18" s="67"/>
       <c r="J18" s="12"/>
       <c r="K18" s="14"/>
     </row>
@@ -2342,7 +2347,7 @@
       <c r="H19" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="I19" s="64"/>
+      <c r="I19" s="67"/>
       <c r="J19" s="12"/>
       <c r="K19" s="14"/>
     </row>
@@ -2363,7 +2368,7 @@
       <c r="H20" s="39" t="s">
         <v>103</v>
       </c>
-      <c r="I20" s="65"/>
+      <c r="I20" s="68"/>
       <c r="J20" s="13"/>
       <c r="K20" s="15"/>
     </row>
@@ -2392,7 +2397,7 @@
       <c r="H21" s="37" t="s">
         <v>35</v>
       </c>
-      <c r="I21" s="71" t="s">
+      <c r="I21" s="60" t="s">
         <v>141</v>
       </c>
       <c r="J21" s="12">
@@ -2419,7 +2424,7 @@
       <c r="H22" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="I22" s="72"/>
+      <c r="I22" s="61"/>
       <c r="J22" s="12">
         <v>4</v>
       </c>
@@ -2442,7 +2447,7 @@
       <c r="H23" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="I23" s="72"/>
+      <c r="I23" s="61"/>
       <c r="J23" s="12">
         <v>3</v>
       </c>
@@ -2465,7 +2470,7 @@
       <c r="H24" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="I24" s="72"/>
+      <c r="I24" s="61"/>
       <c r="J24" s="12">
         <v>2</v>
       </c>
@@ -2488,7 +2493,7 @@
       <c r="H25" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="I25" s="73"/>
+      <c r="I25" s="62"/>
       <c r="J25" s="13">
         <v>1</v>
       </c>
@@ -2521,7 +2526,7 @@
       <c r="H26" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="I26" s="71" t="s">
+      <c r="I26" s="60" t="s">
         <v>106</v>
       </c>
       <c r="J26" s="12">
@@ -2548,7 +2553,7 @@
       <c r="H27" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="I27" s="72"/>
+      <c r="I27" s="61"/>
       <c r="J27" s="12">
         <v>4</v>
       </c>
@@ -2571,7 +2576,7 @@
       <c r="H28" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="I28" s="72"/>
+      <c r="I28" s="61"/>
       <c r="J28" s="12">
         <v>3</v>
       </c>
@@ -2594,7 +2599,7 @@
       <c r="H29" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="I29" s="72"/>
+      <c r="I29" s="61"/>
       <c r="J29" s="12">
         <v>2</v>
       </c>
@@ -2617,7 +2622,7 @@
       <c r="H30" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="I30" s="73"/>
+      <c r="I30" s="62"/>
       <c r="J30" s="13">
         <v>1</v>
       </c>
@@ -2650,7 +2655,7 @@
       <c r="H31" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="I31" s="71" t="s">
+      <c r="I31" s="60" t="s">
         <v>143</v>
       </c>
       <c r="J31" s="12">
@@ -2677,7 +2682,7 @@
       <c r="H32" s="35" t="s">
         <v>110</v>
       </c>
-      <c r="I32" s="72"/>
+      <c r="I32" s="61"/>
       <c r="J32" s="12">
         <v>4</v>
       </c>
@@ -2702,7 +2707,7 @@
       <c r="H33" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="I33" s="72"/>
+      <c r="I33" s="61"/>
       <c r="J33" s="12">
         <v>3</v>
       </c>
@@ -2727,7 +2732,7 @@
       <c r="H34" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="I34" s="72"/>
+      <c r="I34" s="61"/>
       <c r="J34" s="12">
         <v>2</v>
       </c>
@@ -2752,7 +2757,7 @@
       <c r="H35" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="I35" s="73"/>
+      <c r="I35" s="62"/>
       <c r="J35" s="13">
         <v>1</v>
       </c>
@@ -2785,7 +2790,7 @@
       <c r="H36" s="37" t="s">
         <v>51</v>
       </c>
-      <c r="I36" s="71" t="s">
+      <c r="I36" s="60" t="s">
         <v>144</v>
       </c>
       <c r="J36" s="12">
@@ -2812,7 +2817,7 @@
       <c r="H37" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="I37" s="72"/>
+      <c r="I37" s="61"/>
       <c r="J37" s="12">
         <v>4</v>
       </c>
@@ -2835,7 +2840,7 @@
       <c r="H38" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="I38" s="72"/>
+      <c r="I38" s="61"/>
       <c r="J38" s="12">
         <v>3</v>
       </c>
@@ -2858,7 +2863,7 @@
       <c r="H39" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="I39" s="72"/>
+      <c r="I39" s="61"/>
       <c r="J39" s="12">
         <v>2</v>
       </c>
@@ -2881,7 +2886,7 @@
       <c r="H40" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="I40" s="73"/>
+      <c r="I40" s="62"/>
       <c r="J40" s="13">
         <v>1</v>
       </c>
@@ -2914,7 +2919,7 @@
       <c r="H41" s="37" t="s">
         <v>59</v>
       </c>
-      <c r="I41" s="71" t="s">
+      <c r="I41" s="60" t="s">
         <v>114</v>
       </c>
       <c r="J41" s="12">
@@ -2941,7 +2946,7 @@
       <c r="H42" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="I42" s="72"/>
+      <c r="I42" s="61"/>
       <c r="J42" s="12">
         <v>4</v>
       </c>
@@ -2964,7 +2969,7 @@
       <c r="H43" s="35" t="s">
         <v>61</v>
       </c>
-      <c r="I43" s="72"/>
+      <c r="I43" s="61"/>
       <c r="J43" s="12">
         <v>3</v>
       </c>
@@ -2987,7 +2992,7 @@
       <c r="H44" s="35" t="s">
         <v>62</v>
       </c>
-      <c r="I44" s="72"/>
+      <c r="I44" s="61"/>
       <c r="J44" s="12">
         <v>2</v>
       </c>
@@ -3010,7 +3015,7 @@
       <c r="H45" s="36" t="s">
         <v>63</v>
       </c>
-      <c r="I45" s="73"/>
+      <c r="I45" s="62"/>
       <c r="J45" s="13">
         <v>1</v>
       </c>
@@ -3043,7 +3048,7 @@
       <c r="H46" s="33" t="s">
         <v>115</v>
       </c>
-      <c r="I46" s="63" t="s">
+      <c r="I46" s="66" t="s">
         <v>145</v>
       </c>
       <c r="J46" s="12">
@@ -3070,7 +3075,7 @@
       <c r="H47" s="33" t="s">
         <v>116</v>
       </c>
-      <c r="I47" s="64"/>
+      <c r="I47" s="67"/>
       <c r="J47" s="12">
         <v>4</v>
       </c>
@@ -3093,7 +3098,7 @@
       <c r="H48" s="33" t="s">
         <v>117</v>
       </c>
-      <c r="I48" s="64"/>
+      <c r="I48" s="67"/>
       <c r="J48" s="12">
         <v>3</v>
       </c>
@@ -3116,7 +3121,7 @@
       <c r="H49" s="33" t="s">
         <v>118</v>
       </c>
-      <c r="I49" s="64"/>
+      <c r="I49" s="67"/>
       <c r="J49" s="12">
         <v>2</v>
       </c>
@@ -3139,7 +3144,7 @@
       <c r="H50" s="34" t="s">
         <v>119</v>
       </c>
-      <c r="I50" s="65"/>
+      <c r="I50" s="68"/>
       <c r="J50" s="13">
         <v>1</v>
       </c>
@@ -3301,7 +3306,7 @@
       <c r="H56" s="37" t="s">
         <v>152</v>
       </c>
-      <c r="I56" s="71" t="s">
+      <c r="I56" s="60" t="s">
         <v>153</v>
       </c>
       <c r="J56" s="12">
@@ -3328,7 +3333,7 @@
       <c r="H57" s="37" t="s">
         <v>152</v>
       </c>
-      <c r="I57" s="72"/>
+      <c r="I57" s="61"/>
       <c r="J57" s="12">
         <v>4</v>
       </c>
@@ -3353,7 +3358,7 @@
       <c r="H58" s="37" t="s">
         <v>152</v>
       </c>
-      <c r="I58" s="72"/>
+      <c r="I58" s="61"/>
       <c r="J58" s="12">
         <v>3</v>
       </c>
@@ -3378,7 +3383,7 @@
       <c r="H59" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="I59" s="72"/>
+      <c r="I59" s="61"/>
       <c r="J59" s="12">
         <v>2</v>
       </c>
@@ -3403,7 +3408,7 @@
       <c r="H60" s="19" t="s">
         <v>152</v>
       </c>
-      <c r="I60" s="73"/>
+      <c r="I60" s="62"/>
       <c r="J60" s="13">
         <v>1</v>
       </c>
@@ -3436,7 +3441,7 @@
       <c r="H61" s="40" t="s">
         <v>148</v>
       </c>
-      <c r="I61" s="71" t="s">
+      <c r="I61" s="60" t="s">
         <v>149</v>
       </c>
       <c r="J61" s="12">
@@ -3463,7 +3468,7 @@
       <c r="H62" s="40" t="s">
         <v>148</v>
       </c>
-      <c r="I62" s="72"/>
+      <c r="I62" s="61"/>
       <c r="J62" s="12">
         <v>4</v>
       </c>
@@ -3488,7 +3493,7 @@
       <c r="H63" s="40" t="s">
         <v>148</v>
       </c>
-      <c r="I63" s="72"/>
+      <c r="I63" s="61"/>
       <c r="J63" s="12">
         <v>3</v>
       </c>
@@ -3513,7 +3518,7 @@
       <c r="H64" s="40" t="s">
         <v>148</v>
       </c>
-      <c r="I64" s="72"/>
+      <c r="I64" s="61"/>
       <c r="J64" s="12">
         <v>2</v>
       </c>
@@ -3571,7 +3576,7 @@
       <c r="H66" s="40" t="s">
         <v>150</v>
       </c>
-      <c r="I66" s="63" t="s">
+      <c r="I66" s="66" t="s">
         <v>151</v>
       </c>
       <c r="J66" s="12">
@@ -3598,7 +3603,7 @@
       <c r="H67" s="42" t="s">
         <v>137</v>
       </c>
-      <c r="I67" s="64"/>
+      <c r="I67" s="67"/>
       <c r="J67" s="12">
         <v>4</v>
       </c>
@@ -3621,7 +3626,7 @@
       <c r="H68" s="43" t="s">
         <v>128</v>
       </c>
-      <c r="I68" s="64"/>
+      <c r="I68" s="67"/>
       <c r="J68" s="12">
         <v>3</v>
       </c>
@@ -3644,7 +3649,7 @@
       <c r="H69" s="43" t="s">
         <v>129</v>
       </c>
-      <c r="I69" s="64"/>
+      <c r="I69" s="67"/>
       <c r="J69" s="12">
         <v>2</v>
       </c>
@@ -3667,7 +3672,7 @@
       <c r="H70" s="44" t="s">
         <v>130</v>
       </c>
-      <c r="I70" s="65"/>
+      <c r="I70" s="68"/>
       <c r="J70" s="13">
         <v>1</v>
       </c>
@@ -3700,7 +3705,7 @@
       <c r="H71" s="43" t="s">
         <v>131</v>
       </c>
-      <c r="I71" s="63" t="s">
+      <c r="I71" s="66" t="s">
         <v>154</v>
       </c>
       <c r="J71" s="12">
@@ -3727,7 +3732,7 @@
       <c r="H72" s="43" t="s">
         <v>131</v>
       </c>
-      <c r="I72" s="64"/>
+      <c r="I72" s="67"/>
       <c r="J72" s="12">
         <v>4</v>
       </c>
@@ -3752,7 +3757,7 @@
       <c r="H73" s="43" t="s">
         <v>131</v>
       </c>
-      <c r="I73" s="64"/>
+      <c r="I73" s="67"/>
       <c r="J73" s="12">
         <v>3</v>
       </c>
@@ -3777,7 +3782,7 @@
       <c r="H74" s="43" t="s">
         <v>131</v>
       </c>
-      <c r="I74" s="64"/>
+      <c r="I74" s="67"/>
       <c r="J74" s="12">
         <v>2</v>
       </c>
@@ -3802,7 +3807,7 @@
       <c r="H75" s="44" t="s">
         <v>131</v>
       </c>
-      <c r="I75" s="65"/>
+      <c r="I75" s="68"/>
       <c r="J75" s="13">
         <v>1</v>
       </c>
@@ -3835,7 +3840,7 @@
       <c r="H76" s="37" t="s">
         <v>155</v>
       </c>
-      <c r="I76" s="71" t="s">
+      <c r="I76" s="60" t="s">
         <v>160</v>
       </c>
       <c r="J76" s="12">
@@ -3862,7 +3867,7 @@
       <c r="H77" s="35" t="s">
         <v>156</v>
       </c>
-      <c r="I77" s="72"/>
+      <c r="I77" s="61"/>
       <c r="J77" s="12">
         <v>4</v>
       </c>
@@ -3887,7 +3892,7 @@
       <c r="H78" s="35" t="s">
         <v>157</v>
       </c>
-      <c r="I78" s="72"/>
+      <c r="I78" s="61"/>
       <c r="J78" s="12">
         <v>3</v>
       </c>
@@ -3912,7 +3917,7 @@
       <c r="H79" s="35" t="s">
         <v>158</v>
       </c>
-      <c r="I79" s="72"/>
+      <c r="I79" s="61"/>
       <c r="J79" s="12">
         <v>2</v>
       </c>
@@ -3937,7 +3942,7 @@
       <c r="H80" s="36" t="s">
         <v>159</v>
       </c>
-      <c r="I80" s="73"/>
+      <c r="I80" s="62"/>
       <c r="J80" s="13">
         <v>1</v>
       </c>
@@ -3970,14 +3975,14 @@
       <c r="H81" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="I81" s="63" t="s">
+      <c r="I81" s="66" t="s">
         <v>161</v>
       </c>
       <c r="J81" s="12">
         <v>5</v>
       </c>
       <c r="K81" s="14" t="s">
-        <v>104</v>
+        <v>171</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.3">
@@ -3997,7 +4002,7 @@
       <c r="H82" s="35" t="s">
         <v>87</v>
       </c>
-      <c r="I82" s="64"/>
+      <c r="I82" s="67"/>
       <c r="J82" s="12">
         <v>4</v>
       </c>
@@ -4020,7 +4025,7 @@
       <c r="H83" s="35" t="s">
         <v>88</v>
       </c>
-      <c r="I83" s="64"/>
+      <c r="I83" s="67"/>
       <c r="J83" s="12">
         <v>3</v>
       </c>
@@ -4043,7 +4048,7 @@
       <c r="H84" s="35" t="s">
         <v>89</v>
       </c>
-      <c r="I84" s="64"/>
+      <c r="I84" s="67"/>
       <c r="J84" s="12">
         <v>2</v>
       </c>
@@ -4066,28 +4071,28 @@
       <c r="H85" s="45" t="s">
         <v>90</v>
       </c>
-      <c r="I85" s="64"/>
+      <c r="I85" s="67"/>
       <c r="J85" s="12">
         <v>1</v>
       </c>
       <c r="K85" s="14" t="s">
-        <v>105</v>
+        <v>172</v>
       </c>
     </row>
     <row r="86" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A86" s="60" t="s">
+      <c r="A86" s="63" t="s">
         <v>132</v>
       </c>
-      <c r="B86" s="61"/>
-      <c r="C86" s="61"/>
-      <c r="D86" s="61"/>
-      <c r="E86" s="61"/>
-      <c r="F86" s="61"/>
-      <c r="G86" s="61"/>
-      <c r="H86" s="61"/>
-      <c r="I86" s="61"/>
-      <c r="J86" s="61"/>
-      <c r="K86" s="62"/>
+      <c r="B86" s="64"/>
+      <c r="C86" s="64"/>
+      <c r="D86" s="64"/>
+      <c r="E86" s="64"/>
+      <c r="F86" s="64"/>
+      <c r="G86" s="64"/>
+      <c r="H86" s="64"/>
+      <c r="I86" s="64"/>
+      <c r="J86" s="64"/>
+      <c r="K86" s="65"/>
     </row>
     <row r="87" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A87" s="21" t="s">
@@ -4114,7 +4119,7 @@
       <c r="H87" s="24" t="s">
         <v>136</v>
       </c>
-      <c r="I87" s="66" t="s">
+      <c r="I87" s="69" t="s">
         <v>162</v>
       </c>
       <c r="J87" s="25">
@@ -4138,7 +4143,7 @@
       <c r="H88" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="I88" s="67"/>
+      <c r="I88" s="70"/>
       <c r="J88" s="12">
         <v>4</v>
       </c>
@@ -4160,7 +4165,7 @@
       <c r="H89" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="I89" s="67"/>
+      <c r="I89" s="70"/>
       <c r="J89" s="12">
         <v>3</v>
       </c>
@@ -4182,7 +4187,7 @@
       <c r="H90" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="I90" s="67"/>
+      <c r="I90" s="70"/>
       <c r="J90" s="12">
         <v>2</v>
       </c>
@@ -4207,7 +4212,7 @@
       <c r="H91" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="I91" s="68"/>
+      <c r="I91" s="71"/>
       <c r="J91" s="13">
         <v>1</v>
       </c>
@@ -4217,6 +4222,7 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="I11:I15"/>
     <mergeCell ref="I21:I25"/>
     <mergeCell ref="I26:I30"/>
     <mergeCell ref="I31:I35"/>
@@ -4235,7 +4241,6 @@
     <mergeCell ref="I56:I60"/>
     <mergeCell ref="I61:I65"/>
     <mergeCell ref="I6:I10"/>
-    <mergeCell ref="I11:I15"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H51" r:id="rId1" xr:uid="{87B608CB-B79B-4CEE-A3E2-6793DD0064F4}"/>
@@ -4359,7 +4364,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E2C868A-3297-4BC9-A072-2BA55D04EA50}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -4374,7 +4379,7 @@
       <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="79">
+      <c r="B2">
         <v>1</v>
       </c>
     </row>
@@ -4382,7 +4387,7 @@
       <c r="A3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="79">
+      <c r="B3">
         <v>2</v>
       </c>
     </row>
@@ -4390,7 +4395,7 @@
       <c r="A4" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="79">
+      <c r="B4">
         <v>3</v>
       </c>
     </row>
@@ -4398,7 +4403,7 @@
       <c r="A5" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="79">
+      <c r="B5">
         <v>4</v>
       </c>
     </row>
@@ -4406,12 +4411,9 @@
       <c r="A6" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="79">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B7" s="79"/>
+      <c r="B6">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5107,13 +5109,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26BD1FD4-CBF2-4FF9-A9D4-CFE5116A5DD7}">
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="18" width="13" style="54" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A1" s="54" t="s">
         <v>21</v>
       </c>
@@ -5169,7 +5171,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -5182,7 +5184,7 @@
       </c>
       <c r="D2" s="54">
         <f>'Site Selector Data - edited'!G11</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E2" s="54">
         <f>'Site Selector Data - edited'!G16</f>
@@ -5240,8 +5242,16 @@
         <f>'Site Selector Data - edited'!G81</f>
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="T2">
+        <f>AVERAGE(C2:E2)</f>
+        <v>3.3333333333333335</v>
+      </c>
+      <c r="U2">
+        <f>SUM(C2:E2)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -5254,7 +5264,7 @@
       </c>
       <c r="D3" s="54">
         <f>'Site Selector Data - edited'!G12</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E3" s="54">
         <f>'Site Selector Data - edited'!G17</f>
@@ -5312,8 +5322,12 @@
         <f>'Site Selector Data - edited'!G82</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="T3">
+        <f t="shared" ref="T3:T6" si="0">AVERAGE(C3:E3)</f>
+        <v>4.666666666666667</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -5326,7 +5340,7 @@
       </c>
       <c r="D4" s="54">
         <f>'Site Selector Data - edited'!G13</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E4" s="54">
         <f>'Site Selector Data - edited'!G18</f>
@@ -5384,8 +5398,12 @@
         <f>'Site Selector Data - edited'!G83</f>
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="T4">
+        <f t="shared" si="0"/>
+        <v>3.3333333333333335</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -5456,8 +5474,12 @@
         <f>'Site Selector Data - edited'!G84</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="T5">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -5470,7 +5492,7 @@
       </c>
       <c r="D6" s="54">
         <f>'Site Selector Data - edited'!G15</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E6" s="54">
         <f>'Site Selector Data - edited'!G20</f>
@@ -5527,6 +5549,10 @@
       <c r="R6" s="54">
         <f>'Site Selector Data - edited'!G85</f>
         <v>1</v>
+      </c>
+      <c r="T6">
+        <f t="shared" si="0"/>
+        <v>3.3333333333333335</v>
       </c>
     </row>
   </sheetData>
@@ -6061,7 +6087,7 @@
       </c>
       <c r="D7" t="str">
         <f>'Site Selector Data - edited'!K11</f>
-        <v>dryest</v>
+        <v>wettest</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -6106,7 +6132,7 @@
       </c>
       <c r="D11" t="str">
         <f>'Site Selector Data - edited'!K15</f>
-        <v>wettest</v>
+        <v>dryest</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -6915,7 +6941,7 @@
       </c>
       <c r="D77" t="str">
         <f>'Site Selector Data - edited'!K81</f>
-        <v>lowest</v>
+        <v>best</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
feat(ui): sync defaults, category sources from workbook, UX polish
</commit_message>
<xml_diff>
--- a/data/Data_Center_Site_Selector_RH.xlsx
+++ b/data/Data_Center_Site_Selector_RH.xlsx
@@ -8,10 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://colostate-my.sharepoint.com/personal/laffite_colostate_edu/Documents/Desktop/Classes/2026 Spring/CIVE-580C4 Applying AI in Environmental Engr Practice/Final project/App_v2/Siteworks2/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1151" documentId="11_CB780128D071F47F630230D6525DCE3A2746A58A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{021857B9-811B-4D0E-A50C-2B3CD42429A0}"/>
+  <xr:revisionPtr revIDLastSave="1153" documentId="11_CB780128D071F47F630230D6525DCE3A2746A58A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E0319C0-6B49-4D6F-BB71-F3DAD2381B4C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" tabRatio="707" activeTab="4" xr2:uid="{C789D543-12B0-4242-A688-B41AF874B720}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Site Selector Data - edited" sheetId="2" r:id="rId1"/>
@@ -5109,13 +5108,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26BD1FD4-CBF2-4FF9-A9D4-CFE5116A5DD7}">
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="18" width="13" style="54" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A1" s="54" t="s">
         <v>21</v>
       </c>
@@ -5171,7 +5170,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -5242,16 +5241,8 @@
         <f>'Site Selector Data - edited'!G81</f>
         <v>4</v>
       </c>
-      <c r="T2">
-        <f>AVERAGE(C2:E2)</f>
-        <v>3.3333333333333335</v>
-      </c>
-      <c r="U2">
-        <f>SUM(C2:E2)</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -5322,12 +5313,8 @@
         <f>'Site Selector Data - edited'!G82</f>
         <v>2</v>
       </c>
-      <c r="T3">
-        <f t="shared" ref="T3:T6" si="0">AVERAGE(C3:E3)</f>
-        <v>4.666666666666667</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -5398,12 +5385,8 @@
         <f>'Site Selector Data - edited'!G83</f>
         <v>3</v>
       </c>
-      <c r="T4">
-        <f t="shared" si="0"/>
-        <v>3.3333333333333335</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -5474,12 +5457,8 @@
         <f>'Site Selector Data - edited'!G84</f>
         <v>5</v>
       </c>
-      <c r="T5">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -5549,10 +5528,6 @@
       <c r="R6" s="54">
         <f>'Site Selector Data - edited'!G85</f>
         <v>1</v>
-      </c>
-      <c r="T6">
-        <f t="shared" si="0"/>
-        <v>3.3333333333333335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>